<commit_message>
Replace the difficulty-leaking demo text in both question banks
The demo questions read "Hard Question 1: ...", so a paper announced each
question's difficulty to the student. Both banks now carry topic-varied business
questions with no difficulty word in the text; the banks agree on shared question
numbers, and every question text is distinct so the text-matching fallback stays
sound.

question_no, answer and difficulty are untouched. The correct option is placed at
whichever letter the bank already recorded, so allocations and scores are
unaffected: output/question_papers.xlsx is rewritten with the new text but the
exact same sets, and the pinned regression metrics still hold.

Reusing one open workbook across set sheets takes the suite from 296s to 13s —
printing QCd moved the header off row 1, so every sheet was being parsed twice.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/question_bank.xlsx
+++ b/input/question_bank.xlsx
@@ -40,1054 +40,1054 @@
     <t>difficulty</t>
   </si>
   <si>
-    <t>Hard Question 1: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 2: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 3: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 4: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 5: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 6: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 7: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 8: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 9: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 10: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 11: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Hard Question 12: What is the solution to this complex problem?</t>
-  </si>
-  <si>
-    <t>Medium Question 1: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 2: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 3: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 4: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 5: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 6: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 7: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 8: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 9: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 10: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 11: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 12: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 13: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 14: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 15: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 16: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 17: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 18: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 19: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 20: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 21: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 22: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 23: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 24: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 25: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 26: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 27: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 28: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 29: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Medium Question 30: Calculate the following expression.</t>
-  </si>
-  <si>
-    <t>Easy Question 1: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 2: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 3: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 4: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 5: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 6: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 7: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 8: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 9: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 10: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 11: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 12: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 13: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 14: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 15: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 16: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 17: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 18: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 19: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 20: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 21: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 22: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 23: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 24: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 25: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 26: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 27: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Easy Question 28: What is the basic definition of this term?</t>
-  </si>
-  <si>
-    <t>Hard option A1</t>
-  </si>
-  <si>
-    <t>Hard option A2</t>
-  </si>
-  <si>
-    <t>Hard option A3</t>
-  </si>
-  <si>
-    <t>Hard option A4</t>
-  </si>
-  <si>
-    <t>Hard option A5</t>
-  </si>
-  <si>
-    <t>Hard option A6</t>
-  </si>
-  <si>
-    <t>Hard option A7</t>
-  </si>
-  <si>
-    <t>Hard option A8</t>
-  </si>
-  <si>
-    <t>Hard option A9</t>
-  </si>
-  <si>
-    <t>Hard option A10</t>
-  </si>
-  <si>
-    <t>Hard option A11</t>
-  </si>
-  <si>
-    <t>Hard option A12</t>
-  </si>
-  <si>
-    <t>Medium option A1</t>
-  </si>
-  <si>
-    <t>Medium option A2</t>
-  </si>
-  <si>
-    <t>Medium option A3</t>
-  </si>
-  <si>
-    <t>Medium option A4</t>
-  </si>
-  <si>
-    <t>Medium option A5</t>
-  </si>
-  <si>
-    <t>Medium option A6</t>
-  </si>
-  <si>
-    <t>Medium option A7</t>
-  </si>
-  <si>
-    <t>Medium option A8</t>
-  </si>
-  <si>
-    <t>Medium option A9</t>
-  </si>
-  <si>
-    <t>Medium option A10</t>
-  </si>
-  <si>
-    <t>Medium option A11</t>
-  </si>
-  <si>
-    <t>Medium option A12</t>
-  </si>
-  <si>
-    <t>Medium option A13</t>
-  </si>
-  <si>
-    <t>Medium option A14</t>
-  </si>
-  <si>
-    <t>Medium option A15</t>
-  </si>
-  <si>
-    <t>Medium option A16</t>
-  </si>
-  <si>
-    <t>Medium option A17</t>
-  </si>
-  <si>
-    <t>Medium option A18</t>
-  </si>
-  <si>
-    <t>Medium option A19</t>
-  </si>
-  <si>
-    <t>Medium option A20</t>
-  </si>
-  <si>
-    <t>Medium option A21</t>
-  </si>
-  <si>
-    <t>Medium option A22</t>
-  </si>
-  <si>
-    <t>Medium option A23</t>
-  </si>
-  <si>
-    <t>Medium option A24</t>
-  </si>
-  <si>
-    <t>Medium option A25</t>
-  </si>
-  <si>
-    <t>Medium option A26</t>
-  </si>
-  <si>
-    <t>Medium option A27</t>
-  </si>
-  <si>
-    <t>Medium option A28</t>
-  </si>
-  <si>
-    <t>Medium option A29</t>
-  </si>
-  <si>
-    <t>Medium option A30</t>
-  </si>
-  <si>
-    <t>Easy option A1</t>
-  </si>
-  <si>
-    <t>Easy option A2</t>
-  </si>
-  <si>
-    <t>Easy option A3</t>
-  </si>
-  <si>
-    <t>Easy option A4</t>
-  </si>
-  <si>
-    <t>Easy option A5</t>
-  </si>
-  <si>
-    <t>Easy option A6</t>
-  </si>
-  <si>
-    <t>Easy option A7</t>
-  </si>
-  <si>
-    <t>Easy option A8</t>
-  </si>
-  <si>
-    <t>Easy option A9</t>
-  </si>
-  <si>
-    <t>Easy option A10</t>
-  </si>
-  <si>
-    <t>Easy option A11</t>
-  </si>
-  <si>
-    <t>Easy option A12</t>
-  </si>
-  <si>
-    <t>Easy option A13</t>
-  </si>
-  <si>
-    <t>Easy option A14</t>
-  </si>
-  <si>
-    <t>Easy option A15</t>
-  </si>
-  <si>
-    <t>Easy option A16</t>
-  </si>
-  <si>
-    <t>Easy option A17</t>
-  </si>
-  <si>
-    <t>Easy option A18</t>
-  </si>
-  <si>
-    <t>Easy option A19</t>
-  </si>
-  <si>
-    <t>Easy option A20</t>
-  </si>
-  <si>
-    <t>Easy option A21</t>
-  </si>
-  <si>
-    <t>Easy option A22</t>
-  </si>
-  <si>
-    <t>Easy option A23</t>
-  </si>
-  <si>
-    <t>Easy option A24</t>
-  </si>
-  <si>
-    <t>Easy option A25</t>
-  </si>
-  <si>
-    <t>Easy option A26</t>
-  </si>
-  <si>
-    <t>Easy option A27</t>
-  </si>
-  <si>
-    <t>Easy option A28</t>
-  </si>
-  <si>
-    <t>Hard option B1</t>
-  </si>
-  <si>
-    <t>Hard option B2</t>
-  </si>
-  <si>
-    <t>Hard option B3</t>
-  </si>
-  <si>
-    <t>Hard option B4</t>
-  </si>
-  <si>
-    <t>Hard option B5</t>
-  </si>
-  <si>
-    <t>Hard option B6</t>
-  </si>
-  <si>
-    <t>Hard option B7</t>
-  </si>
-  <si>
-    <t>Hard option B8</t>
-  </si>
-  <si>
-    <t>Hard option B9</t>
-  </si>
-  <si>
-    <t>Hard option B10</t>
-  </si>
-  <si>
-    <t>Hard option B11</t>
-  </si>
-  <si>
-    <t>Hard option B12</t>
-  </si>
-  <si>
-    <t>Medium option B1</t>
-  </si>
-  <si>
-    <t>Medium option B2</t>
-  </si>
-  <si>
-    <t>Medium option B3</t>
-  </si>
-  <si>
-    <t>Medium option B4</t>
-  </si>
-  <si>
-    <t>Medium option B5</t>
-  </si>
-  <si>
-    <t>Medium option B6</t>
-  </si>
-  <si>
-    <t>Medium option B7</t>
-  </si>
-  <si>
-    <t>Medium option B8</t>
-  </si>
-  <si>
-    <t>Medium option B9</t>
-  </si>
-  <si>
-    <t>Medium option B10</t>
-  </si>
-  <si>
-    <t>Medium option B11</t>
-  </si>
-  <si>
-    <t>Medium option B12</t>
-  </si>
-  <si>
-    <t>Medium option B13</t>
-  </si>
-  <si>
-    <t>Medium option B14</t>
-  </si>
-  <si>
-    <t>Medium option B15</t>
-  </si>
-  <si>
-    <t>Medium option B16</t>
-  </si>
-  <si>
-    <t>Medium option B17</t>
-  </si>
-  <si>
-    <t>Medium option B18</t>
-  </si>
-  <si>
-    <t>Medium option B19</t>
-  </si>
-  <si>
-    <t>Medium option B20</t>
-  </si>
-  <si>
-    <t>Medium option B21</t>
-  </si>
-  <si>
-    <t>Medium option B22</t>
-  </si>
-  <si>
-    <t>Medium option B23</t>
-  </si>
-  <si>
-    <t>Medium option B24</t>
-  </si>
-  <si>
-    <t>Medium option B25</t>
-  </si>
-  <si>
-    <t>Medium option B26</t>
-  </si>
-  <si>
-    <t>Medium option B27</t>
-  </si>
-  <si>
-    <t>Medium option B28</t>
-  </si>
-  <si>
-    <t>Medium option B29</t>
-  </si>
-  <si>
-    <t>Medium option B30</t>
-  </si>
-  <si>
-    <t>Easy option B1</t>
-  </si>
-  <si>
-    <t>Easy option B2</t>
-  </si>
-  <si>
-    <t>Easy option B3</t>
-  </si>
-  <si>
-    <t>Easy option B4</t>
-  </si>
-  <si>
-    <t>Easy option B5</t>
-  </si>
-  <si>
-    <t>Easy option B6</t>
-  </si>
-  <si>
-    <t>Easy option B7</t>
-  </si>
-  <si>
-    <t>Easy option B8</t>
-  </si>
-  <si>
-    <t>Easy option B9</t>
-  </si>
-  <si>
-    <t>Easy option B10</t>
-  </si>
-  <si>
-    <t>Easy option B11</t>
-  </si>
-  <si>
-    <t>Easy option B12</t>
-  </si>
-  <si>
-    <t>Easy option B13</t>
-  </si>
-  <si>
-    <t>Easy option B14</t>
-  </si>
-  <si>
-    <t>Easy option B15</t>
-  </si>
-  <si>
-    <t>Easy option B16</t>
-  </si>
-  <si>
-    <t>Easy option B17</t>
-  </si>
-  <si>
-    <t>Easy option B18</t>
-  </si>
-  <si>
-    <t>Easy option B19</t>
-  </si>
-  <si>
-    <t>Easy option B20</t>
-  </si>
-  <si>
-    <t>Easy option B21</t>
-  </si>
-  <si>
-    <t>Easy option B22</t>
-  </si>
-  <si>
-    <t>Easy option B23</t>
-  </si>
-  <si>
-    <t>Easy option B24</t>
-  </si>
-  <si>
-    <t>Easy option B25</t>
-  </si>
-  <si>
-    <t>Easy option B26</t>
-  </si>
-  <si>
-    <t>Easy option B27</t>
-  </si>
-  <si>
-    <t>Easy option B28</t>
-  </si>
-  <si>
-    <t>Hard option C1</t>
-  </si>
-  <si>
-    <t>Hard option C2</t>
-  </si>
-  <si>
-    <t>Hard option C3</t>
-  </si>
-  <si>
-    <t>Hard option C4</t>
-  </si>
-  <si>
-    <t>Hard option C5</t>
-  </si>
-  <si>
-    <t>Hard option C6</t>
-  </si>
-  <si>
-    <t>Hard option C7</t>
-  </si>
-  <si>
-    <t>Hard option C8</t>
-  </si>
-  <si>
-    <t>Hard option C9</t>
-  </si>
-  <si>
-    <t>Hard option C10</t>
-  </si>
-  <si>
-    <t>Hard option C11</t>
-  </si>
-  <si>
-    <t>Hard option C12</t>
-  </si>
-  <si>
-    <t>Medium option C1</t>
-  </si>
-  <si>
-    <t>Medium option C2</t>
-  </si>
-  <si>
-    <t>Medium option C3</t>
-  </si>
-  <si>
-    <t>Medium option C4</t>
-  </si>
-  <si>
-    <t>Medium option C5</t>
-  </si>
-  <si>
-    <t>Medium option C6</t>
-  </si>
-  <si>
-    <t>Medium option C7</t>
-  </si>
-  <si>
-    <t>Medium option C8</t>
-  </si>
-  <si>
-    <t>Medium option C9</t>
-  </si>
-  <si>
-    <t>Medium option C10</t>
-  </si>
-  <si>
-    <t>Medium option C11</t>
-  </si>
-  <si>
-    <t>Medium option C12</t>
-  </si>
-  <si>
-    <t>Medium option C13</t>
-  </si>
-  <si>
-    <t>Medium option C14</t>
-  </si>
-  <si>
-    <t>Medium option C15</t>
-  </si>
-  <si>
-    <t>Medium option C16</t>
-  </si>
-  <si>
-    <t>Medium option C17</t>
-  </si>
-  <si>
-    <t>Medium option C18</t>
-  </si>
-  <si>
-    <t>Medium option C19</t>
-  </si>
-  <si>
-    <t>Medium option C20</t>
-  </si>
-  <si>
-    <t>Medium option C21</t>
-  </si>
-  <si>
-    <t>Medium option C22</t>
-  </si>
-  <si>
-    <t>Medium option C23</t>
-  </si>
-  <si>
-    <t>Medium option C24</t>
-  </si>
-  <si>
-    <t>Medium option C25</t>
-  </si>
-  <si>
-    <t>Medium option C26</t>
-  </si>
-  <si>
-    <t>Medium option C27</t>
-  </si>
-  <si>
-    <t>Medium option C28</t>
-  </si>
-  <si>
-    <t>Medium option C29</t>
-  </si>
-  <si>
-    <t>Medium option C30</t>
-  </si>
-  <si>
-    <t>Easy option C1</t>
-  </si>
-  <si>
-    <t>Easy option C2</t>
-  </si>
-  <si>
-    <t>Easy option C3</t>
-  </si>
-  <si>
-    <t>Easy option C4</t>
-  </si>
-  <si>
-    <t>Easy option C5</t>
-  </si>
-  <si>
-    <t>Easy option C6</t>
-  </si>
-  <si>
-    <t>Easy option C7</t>
-  </si>
-  <si>
-    <t>Easy option C8</t>
-  </si>
-  <si>
-    <t>Easy option C9</t>
-  </si>
-  <si>
-    <t>Easy option C10</t>
-  </si>
-  <si>
-    <t>Easy option C11</t>
-  </si>
-  <si>
-    <t>Easy option C12</t>
-  </si>
-  <si>
-    <t>Easy option C13</t>
-  </si>
-  <si>
-    <t>Easy option C14</t>
-  </si>
-  <si>
-    <t>Easy option C15</t>
-  </si>
-  <si>
-    <t>Easy option C16</t>
-  </si>
-  <si>
-    <t>Easy option C17</t>
-  </si>
-  <si>
-    <t>Easy option C18</t>
-  </si>
-  <si>
-    <t>Easy option C19</t>
-  </si>
-  <si>
-    <t>Easy option C20</t>
-  </si>
-  <si>
-    <t>Easy option C21</t>
-  </si>
-  <si>
-    <t>Easy option C22</t>
-  </si>
-  <si>
-    <t>Easy option C23</t>
-  </si>
-  <si>
-    <t>Easy option C24</t>
-  </si>
-  <si>
-    <t>Easy option C25</t>
-  </si>
-  <si>
-    <t>Easy option C26</t>
-  </si>
-  <si>
-    <t>Easy option C27</t>
-  </si>
-  <si>
-    <t>Easy option C28</t>
-  </si>
-  <si>
-    <t>Hard option D1</t>
-  </si>
-  <si>
-    <t>Hard option D2</t>
-  </si>
-  <si>
-    <t>Hard option D3</t>
-  </si>
-  <si>
-    <t>Hard option D4</t>
-  </si>
-  <si>
-    <t>Hard option D5</t>
-  </si>
-  <si>
-    <t>Hard option D6</t>
-  </si>
-  <si>
-    <t>Hard option D7</t>
-  </si>
-  <si>
-    <t>Hard option D8</t>
-  </si>
-  <si>
-    <t>Hard option D9</t>
-  </si>
-  <si>
-    <t>Hard option D10</t>
-  </si>
-  <si>
-    <t>Hard option D11</t>
-  </si>
-  <si>
-    <t>Hard option D12</t>
-  </si>
-  <si>
-    <t>Medium option D1</t>
-  </si>
-  <si>
-    <t>Medium option D2</t>
-  </si>
-  <si>
-    <t>Medium option D3</t>
-  </si>
-  <si>
-    <t>Medium option D4</t>
-  </si>
-  <si>
-    <t>Medium option D5</t>
-  </si>
-  <si>
-    <t>Medium option D6</t>
-  </si>
-  <si>
-    <t>Medium option D7</t>
-  </si>
-  <si>
-    <t>Medium option D8</t>
-  </si>
-  <si>
-    <t>Medium option D9</t>
-  </si>
-  <si>
-    <t>Medium option D10</t>
-  </si>
-  <si>
-    <t>Medium option D11</t>
-  </si>
-  <si>
-    <t>Medium option D12</t>
-  </si>
-  <si>
-    <t>Medium option D13</t>
-  </si>
-  <si>
-    <t>Medium option D14</t>
-  </si>
-  <si>
-    <t>Medium option D15</t>
-  </si>
-  <si>
-    <t>Medium option D16</t>
-  </si>
-  <si>
-    <t>Medium option D17</t>
-  </si>
-  <si>
-    <t>Medium option D18</t>
-  </si>
-  <si>
-    <t>Medium option D19</t>
-  </si>
-  <si>
-    <t>Medium option D20</t>
-  </si>
-  <si>
-    <t>Medium option D21</t>
-  </si>
-  <si>
-    <t>Medium option D22</t>
-  </si>
-  <si>
-    <t>Medium option D23</t>
-  </si>
-  <si>
-    <t>Medium option D24</t>
-  </si>
-  <si>
-    <t>Medium option D25</t>
-  </si>
-  <si>
-    <t>Medium option D26</t>
-  </si>
-  <si>
-    <t>Medium option D27</t>
-  </si>
-  <si>
-    <t>Medium option D28</t>
-  </si>
-  <si>
-    <t>Medium option D29</t>
-  </si>
-  <si>
-    <t>Medium option D30</t>
-  </si>
-  <si>
-    <t>Easy option D1</t>
-  </si>
-  <si>
-    <t>Easy option D2</t>
-  </si>
-  <si>
-    <t>Easy option D3</t>
-  </si>
-  <si>
-    <t>Easy option D4</t>
-  </si>
-  <si>
-    <t>Easy option D5</t>
-  </si>
-  <si>
-    <t>Easy option D6</t>
-  </si>
-  <si>
-    <t>Easy option D7</t>
-  </si>
-  <si>
-    <t>Easy option D8</t>
-  </si>
-  <si>
-    <t>Easy option D9</t>
-  </si>
-  <si>
-    <t>Easy option D10</t>
-  </si>
-  <si>
-    <t>Easy option D11</t>
-  </si>
-  <si>
-    <t>Easy option D12</t>
-  </si>
-  <si>
-    <t>Easy option D13</t>
-  </si>
-  <si>
-    <t>Easy option D14</t>
-  </si>
-  <si>
-    <t>Easy option D15</t>
-  </si>
-  <si>
-    <t>Easy option D16</t>
-  </si>
-  <si>
-    <t>Easy option D17</t>
-  </si>
-  <si>
-    <t>Easy option D18</t>
-  </si>
-  <si>
-    <t>Easy option D19</t>
-  </si>
-  <si>
-    <t>Easy option D20</t>
-  </si>
-  <si>
-    <t>Easy option D21</t>
-  </si>
-  <si>
-    <t>Easy option D22</t>
-  </si>
-  <si>
-    <t>Easy option D23</t>
-  </si>
-  <si>
-    <t>Easy option D24</t>
-  </si>
-  <si>
-    <t>Easy option D25</t>
-  </si>
-  <si>
-    <t>Easy option D26</t>
-  </si>
-  <si>
-    <t>Easy option D27</t>
-  </si>
-  <si>
-    <t>Easy option D28</t>
+    <t>What is the primary purpose of a SWOT analysis?</t>
+  </si>
+  <si>
+    <t>What does a company's mission statement describe?</t>
+  </si>
+  <si>
+    <t>In a competitive market, what is a barrier to entry?</t>
+  </si>
+  <si>
+    <t>What is meant by economies of scale?</t>
+  </si>
+  <si>
+    <t>What does market segmentation involve?</t>
+  </si>
+  <si>
+    <t>What is a company's value proposition?</t>
+  </si>
+  <si>
+    <t>What is the main function of working capital?</t>
+  </si>
+  <si>
+    <t>What does a break-even point represent?</t>
+  </si>
+  <si>
+    <t>Why do firms diversify into new markets?</t>
+  </si>
+  <si>
+    <t>What is a core competency?</t>
+  </si>
+  <si>
+    <t>What is the role of a board of directors?</t>
+  </si>
+  <si>
+    <t>What does 'first-mover advantage' refer to?</t>
+  </si>
+  <si>
+    <t>What is the purpose of a cash flow forecast?</t>
+  </si>
+  <si>
+    <t>What is brand equity?</t>
+  </si>
+  <si>
+    <t>What does outsourcing typically allow a firm to do?</t>
+  </si>
+  <si>
+    <t>What is a supply chain?</t>
+  </si>
+  <si>
+    <t>What is the aim of benchmarking?</t>
+  </si>
+  <si>
+    <t>What does a merger involve?</t>
+  </si>
+  <si>
+    <t>What is meant by a firm's operating margin?</t>
+  </si>
+  <si>
+    <t>Why is customer retention valuable?</t>
+  </si>
+  <si>
+    <t>What is a stakeholder?</t>
+  </si>
+  <si>
+    <t>What does 'due diligence' mean ahead of an acquisition?</t>
+  </si>
+  <si>
+    <t>What is the purpose of a pilot launch?</t>
+  </si>
+  <si>
+    <t>What is a fixed cost?</t>
+  </si>
+  <si>
+    <t>What does a distribution channel do?</t>
+  </si>
+  <si>
+    <t>Why might a firm license its technology to others?</t>
+  </si>
+  <si>
+    <t>What is the importance of aligning internal capabilities with external opportunities?</t>
+  </si>
+  <si>
+    <t>What does a profit and loss statement show?</t>
+  </si>
+  <si>
+    <t>What is the purpose of market research?</t>
+  </si>
+  <si>
+    <t>What is a competitive advantage?</t>
+  </si>
+  <si>
+    <t>What does inventory turnover measure?</t>
+  </si>
+  <si>
+    <t>Why do organisations use KPIs?</t>
+  </si>
+  <si>
+    <t>What is a joint venture?</t>
+  </si>
+  <si>
+    <t>What is the purpose of a business model?</t>
+  </si>
+  <si>
+    <t>What does 'time to market' measure?</t>
+  </si>
+  <si>
+    <t>Why is cash different from profit?</t>
+  </si>
+  <si>
+    <t>What is a niche market?</t>
+  </si>
+  <si>
+    <t>What does organisational culture refer to?</t>
+  </si>
+  <si>
+    <t>What is the purpose of a budget?</t>
+  </si>
+  <si>
+    <t>What is meant by 'scalability'?</t>
+  </si>
+  <si>
+    <t>Why do firms conduct competitor analysis?</t>
+  </si>
+  <si>
+    <t>What is the role of a supplier contract?</t>
+  </si>
+  <si>
+    <t>What does customer lifetime value estimate?</t>
+  </si>
+  <si>
+    <t>What is a strategic objective?</t>
+  </si>
+  <si>
+    <t>What does 'return on investment' compare?</t>
+  </si>
+  <si>
+    <t>Why is delegation important for a manager?</t>
+  </si>
+  <si>
+    <t>What is a product life cycle?</t>
+  </si>
+  <si>
+    <t>What does 'differentiation' mean as a strategy?</t>
+  </si>
+  <si>
+    <t>What is the purpose of an organisational structure?</t>
+  </si>
+  <si>
+    <t>Why do businesses hold buffer stock?</t>
+  </si>
+  <si>
+    <t>What is meant by 'market share'?</t>
+  </si>
+  <si>
+    <t>What does a feasibility study assess?</t>
+  </si>
+  <si>
+    <t>Why is a diverse team often an advantage?</t>
+  </si>
+  <si>
+    <t>What is 'churn rate'?</t>
+  </si>
+  <si>
+    <t>What is the purpose of quality control?</t>
+  </si>
+  <si>
+    <t>What does 'liquidity' describe?</t>
+  </si>
+  <si>
+    <t>Why might a firm choose a franchise model?</t>
+  </si>
+  <si>
+    <t>What is a target audience?</t>
+  </si>
+  <si>
+    <t>What does 'lead time' mean?</t>
+  </si>
+  <si>
+    <t>Why do companies publish annual reports?</t>
+  </si>
+  <si>
+    <t>What is 'opportunity cost'?</t>
+  </si>
+  <si>
+    <t>What does a Gantt chart display?</t>
+  </si>
+  <si>
+    <t>What is meant by 'vertical integration'?</t>
+  </si>
+  <si>
+    <t>Why is a contingency plan useful?</t>
+  </si>
+  <si>
+    <t>What does 'gross profit' equal?</t>
+  </si>
+  <si>
+    <t>What is the purpose of a service level agreement?</t>
+  </si>
+  <si>
+    <t>Why do firms invest in staff training?</t>
+  </si>
+  <si>
+    <t>What is 'price elasticity of demand'?</t>
+  </si>
+  <si>
+    <t>What does a risk register record?</t>
+  </si>
+  <si>
+    <t>Why is market positioning important?</t>
+  </si>
+  <si>
+    <t>To calculate a company's quarterly tax liability</t>
+  </si>
+  <si>
+    <t>The exact revenue target for the next quarter</t>
+  </si>
+  <si>
+    <t>A tariff paid by existing firms on exports</t>
+  </si>
+  <si>
+    <t>Cost per unit falls as output volume rises</t>
+  </si>
+  <si>
+    <t>Reducing the number of products a firm sells</t>
+  </si>
+  <si>
+    <t>The total book value of its fixed assets</t>
+  </si>
+  <si>
+    <t>To pay long-term shareholder dividends</t>
+  </si>
+  <si>
+    <t>The sales level at which total revenue equals total cost</t>
+  </si>
+  <si>
+    <t>To guarantee a higher share price within a year</t>
+  </si>
+  <si>
+    <t>The department with the largest headcount</t>
+  </si>
+  <si>
+    <t>To handle day-to-day customer complaints</t>
+  </si>
+  <si>
+    <t>The benefit a firm gains by entering a market before its rivals</t>
+  </si>
+  <si>
+    <t>To record historic profits for tax purposes</t>
+  </si>
+  <si>
+    <t>The share of a company owned by its founders</t>
+  </si>
+  <si>
+    <t>Increase the number of shares in issue</t>
+  </si>
+  <si>
+    <t>The network of organisations involved in producing and delivering a product</t>
+  </si>
+  <si>
+    <t>To set the opening price of a new share issue</t>
+  </si>
+  <si>
+    <t>One company lending money to another</t>
+  </si>
+  <si>
+    <t>The gap between the highest and lowest salary</t>
+  </si>
+  <si>
+    <t>Keeping an existing customer usually costs less than winning a new one</t>
+  </si>
+  <si>
+    <t>Only a person who owns shares in the company</t>
+  </si>
+  <si>
+    <t>Announcing the deal to the press in advance</t>
+  </si>
+  <si>
+    <t>To train pilots to operate company aircraft</t>
+  </si>
+  <si>
+    <t>A cost that does not change with the level of output in the short run</t>
+  </si>
+  <si>
+    <t>Sets the manufacturing schedule for a factory</t>
+  </si>
+  <si>
+    <t>To surrender ownership of its patents permanently</t>
+  </si>
+  <si>
+    <t>It is more relevant for small-mid sized startups</t>
+  </si>
+  <si>
+    <t>Revenues and expenses across a defined period</t>
+  </si>
+  <si>
+    <t>To increase the price of an existing product</t>
+  </si>
+  <si>
+    <t>Any product that is cheaper than the average</t>
+  </si>
+  <si>
+    <t>The number of warehouses a firm operates</t>
+  </si>
+  <si>
+    <t>To track progress against objectives using agreed measures</t>
+  </si>
+  <si>
+    <t>A loan made jointly by two banks</t>
+  </si>
+  <si>
+    <t>To list the furniture and equipment owned</t>
+  </si>
+  <si>
+    <t>The opening hours of a retail outlet</t>
+  </si>
+  <si>
+    <t>A firm can record a profit and still lack the cash to pay its bills</t>
+  </si>
+  <si>
+    <t>A market in which prices never change</t>
+  </si>
+  <si>
+    <t>The physical design of the office building</t>
+  </si>
+  <si>
+    <t>To calculate the market value of shares</t>
+  </si>
+  <si>
+    <t>The ability to grow output or users without a proportional rise in cost</t>
+  </si>
+  <si>
+    <t>To agree prices jointly with rivals</t>
+  </si>
+  <si>
+    <t>To transfer ownership of the supplier to the buyer</t>
+  </si>
+  <si>
+    <t>The age of the average customer</t>
+  </si>
+  <si>
+    <t>A daily task assigned to a team member</t>
+  </si>
+  <si>
+    <t>The number of investors against the share price</t>
+  </si>
+  <si>
+    <t>It frees the manager's time and develops the capability of the team</t>
+  </si>
+  <si>
+    <t>The warranty period offered to buyers</t>
+  </si>
+  <si>
+    <t>Charging the lowest price in the market</t>
+  </si>
+  <si>
+    <t>To set the company's annual revenue target</t>
+  </si>
+  <si>
+    <t>To absorb unexpected swings in demand or supply</t>
+  </si>
+  <si>
+    <t>The percentage of a company owned by its founder</t>
+  </si>
+  <si>
+    <t>How satisfied current employees are</t>
+  </si>
+  <si>
+    <t>It reduces the need for team meetings</t>
+  </si>
+  <si>
+    <t>The proportion of customers who stop buying over a given period</t>
+  </si>
+  <si>
+    <t>To increase production speed regardless of defects</t>
+  </si>
+  <si>
+    <t>The volume of goods a firm can store</t>
+  </si>
+  <si>
+    <t>To avoid having to set any brand standards</t>
+  </si>
+  <si>
+    <t>The specific group a product or message is intended to reach</t>
+  </si>
+  <si>
+    <t>The time a manager spends leading meetings</t>
+  </si>
+  <si>
+    <t>To advertise products to new customers</t>
+  </si>
+  <si>
+    <t>The fee charged to enter a new market</t>
+  </si>
+  <si>
+    <t>Project tasks and their durations across a timeline</t>
+  </si>
+  <si>
+    <t>Promoting staff into more senior positions</t>
+  </si>
+  <si>
+    <t>It removes all risk from a project</t>
+  </si>
+  <si>
+    <t>Revenue less every expense including tax</t>
+  </si>
+  <si>
+    <t>To define the standard of service a provider commits to deliver</t>
+  </si>
+  <si>
+    <t>To reduce the number of roles required</t>
+  </si>
+  <si>
+    <t>The range of prices a retailer may legally charge</t>
+  </si>
+  <si>
+    <t>The names of everyone who has taken a loan</t>
+  </si>
+  <si>
+    <t>It shapes how customers perceive an offering relative to alternatives</t>
+  </si>
+  <si>
+    <t>To assess internal strengths and weaknesses alongside external opportunities and threats</t>
+  </si>
+  <si>
+    <t>The legal structure of the shareholding</t>
+  </si>
+  <si>
+    <t>A clause preventing employees from taking leave</t>
+  </si>
+  <si>
+    <t>Prices rise automatically in line with inflation</t>
+  </si>
+  <si>
+    <t>Dividing a broad market into groups of buyers with similar needs</t>
+  </si>
+  <si>
+    <t>The dividend paid per share each year</t>
+  </si>
+  <si>
+    <t>To purchase manufacturing plants outright</t>
+  </si>
+  <si>
+    <t>The point at which a product is withdrawn from sale</t>
+  </si>
+  <si>
+    <t>To reduce dependence on a single source of revenue</t>
+  </si>
+  <si>
+    <t>The oldest product still in the catalogue</t>
+  </si>
+  <si>
+    <t>To approve individual purchase orders</t>
+  </si>
+  <si>
+    <t>The discount offered to the first customer of the day</t>
+  </si>
+  <si>
+    <t>To anticipate when money will enter and leave the business</t>
+  </si>
+  <si>
+    <t>The cost of registering a trademark</t>
+  </si>
+  <si>
+    <t>Avoid paying value-added tax</t>
+  </si>
+  <si>
+    <t>A queue of customers waiting for a service</t>
+  </si>
+  <si>
+    <t>To compare performance against a strong reference point and identify gaps</t>
+  </si>
+  <si>
+    <t>A firm splitting its shares into smaller units</t>
+  </si>
+  <si>
+    <t>The interest rate charged on its overdraft</t>
+  </si>
+  <si>
+    <t>Existing customers are exempt from price increases</t>
+  </si>
+  <si>
+    <t>Any party affected by, or able to affect, the organisation's activities</t>
+  </si>
+  <si>
+    <t>Paying a deposit into the seller's bank account</t>
+  </si>
+  <si>
+    <t>To reduce the product's manufacturing cost</t>
+  </si>
+  <si>
+    <t>A cost that is paid on a fixed date each month</t>
+  </si>
+  <si>
+    <t>Carries a product from producer through to the end customer</t>
+  </si>
+  <si>
+    <t>To avoid publishing its annual accounts</t>
+  </si>
+  <si>
+    <t>It guarantees market share dominance</t>
+  </si>
+  <si>
+    <t>The company's assets at a single moment in time</t>
+  </si>
+  <si>
+    <t>To gather evidence about customer needs and market conditions before deciding</t>
+  </si>
+  <si>
+    <t>The largest advertising budget in the sector</t>
+  </si>
+  <si>
+    <t>The value of stock lost to damage</t>
+  </si>
+  <si>
+    <t>To replace the need for financial accounts</t>
+  </si>
+  <si>
+    <t>A shared enterprise in which two firms pool resources for a specific purpose</t>
+  </si>
+  <si>
+    <t>To record the minutes of board meetings</t>
+  </si>
+  <si>
+    <t>The delay between an order and its payment</t>
+  </si>
+  <si>
+    <t>Profit is always larger than the cash held</t>
+  </si>
+  <si>
+    <t>A narrow, specialised segment with distinct needs</t>
+  </si>
+  <si>
+    <t>The list of public holidays observed</t>
+  </si>
+  <si>
+    <t>To record customer complaints</t>
+  </si>
+  <si>
+    <t>The ability to weigh goods accurately</t>
+  </si>
+  <si>
+    <t>To understand rivals' positions and anticipate their moves</t>
+  </si>
+  <si>
+    <t>To guarantee the supplier's profitability</t>
+  </si>
+  <si>
+    <t>The total profit expected from a customer across the whole relationship</t>
+  </si>
+  <si>
+    <t>A rule about workplace dress code</t>
+  </si>
+  <si>
+    <t>The salary of managers against that of staff</t>
+  </si>
+  <si>
+    <t>It removes the manager's accountability entirely</t>
+  </si>
+  <si>
+    <t>The stages a product passes through from introduction to decline</t>
+  </si>
+  <si>
+    <t>Selling in as many countries as possible</t>
+  </si>
+  <si>
+    <t>To determine the dividend policy</t>
+  </si>
+  <si>
+    <t>To increase the value of the company's shares</t>
+  </si>
+  <si>
+    <t>A firm's sales expressed as a proportion of total market sales</t>
+  </si>
+  <si>
+    <t>The historic accuracy of past accounts</t>
+  </si>
+  <si>
+    <t>It removes the requirement for a manager</t>
+  </si>
+  <si>
+    <t>The speed at which stock moves through a warehouse</t>
+  </si>
+  <si>
+    <t>To ensure output consistently meets defined standards</t>
+  </si>
+  <si>
+    <t>The total value of a company's debt</t>
+  </si>
+  <si>
+    <t>To transfer its tax obligations to others</t>
+  </si>
+  <si>
+    <t>Everyone who has ever visited the website</t>
+  </si>
+  <si>
+    <t>The time between placing an order and receiving it</t>
+  </si>
+  <si>
+    <t>To recruit candidates for vacancies</t>
+  </si>
+  <si>
+    <t>The cost of missed delivery deadlines</t>
+  </si>
+  <si>
+    <t>A company's profits by product line</t>
+  </si>
+  <si>
+    <t>Taking ownership of stages further up or down one's own supply chain</t>
+  </si>
+  <si>
+    <t>It replaces the need for insurance</t>
+  </si>
+  <si>
+    <t>The cash held at the end of the year</t>
+  </si>
+  <si>
+    <t>To set the wages of the provider's staff</t>
+  </si>
+  <si>
+    <t>To build the skills the organisation needs to perform and adapt</t>
+  </si>
+  <si>
+    <t>The speed at which prices are updated</t>
+  </si>
+  <si>
+    <t>Accidents that occurred on site last year</t>
+  </si>
+  <si>
+    <t>It determines where a shop is physically built</t>
+  </si>
+  <si>
+    <t>To schedule production runs across factories</t>
+  </si>
+  <si>
+    <t>The organisation's core purpose and reason for existing</t>
+  </si>
+  <si>
+    <t>A limit on how many products a firm may advertise</t>
+  </si>
+  <si>
+    <t>Staff numbers grow in step with revenue</t>
+  </si>
+  <si>
+    <t>Merging two competing companies</t>
+  </si>
+  <si>
+    <t>The specific benefit it promises to deliver to a chosen customer</t>
+  </si>
+  <si>
+    <t>To settle corporate income tax arrears</t>
+  </si>
+  <si>
+    <t>The maximum output a factory can physically produce</t>
+  </si>
+  <si>
+    <t>To avoid having to file annual accounts</t>
+  </si>
+  <si>
+    <t>A capability a firm performs distinctively well and that rivals struggle to imitate</t>
+  </si>
+  <si>
+    <t>To deliver staff training sessions</t>
+  </si>
+  <si>
+    <t>The right to speak first at a shareholder meeting</t>
+  </si>
+  <si>
+    <t>To place a valuation on the company's brand</t>
+  </si>
+  <si>
+    <t>The commercial value that arises from customer perception of a brand</t>
+  </si>
+  <si>
+    <t>Extend its patent protection period</t>
+  </si>
+  <si>
+    <t>A sequence of managers in a reporting line</t>
+  </si>
+  <si>
+    <t>To calculate depreciation on equipment</t>
+  </si>
+  <si>
+    <t>Two companies combining to form a single entity</t>
+  </si>
+  <si>
+    <t>The proportion of staff working overtime</t>
+  </si>
+  <si>
+    <t>Retained customers reduce a firm's tax bill</t>
+  </si>
+  <si>
+    <t>An employee who has served more than ten years</t>
+  </si>
+  <si>
+    <t>Investigating the target's finances, risks and obligations before committing</t>
+  </si>
+  <si>
+    <t>To register the product's design rights</t>
+  </si>
+  <si>
+    <t>A price agreed with a customer in advance</t>
+  </si>
+  <si>
+    <t>Determines the interest charged on trade credit</t>
+  </si>
+  <si>
+    <t>To earn revenue from the technology without manufacturing it itself</t>
+  </si>
+  <si>
+    <t>It reduces the need for innovation and cost reduction</t>
+  </si>
+  <si>
+    <t>The names of all current shareholders</t>
+  </si>
+  <si>
+    <t>To recruit staff for the sales department</t>
+  </si>
+  <si>
+    <t>Something that lets a firm outperform rivals in a way they struggle to copy</t>
+  </si>
+  <si>
+    <t>The cost of transporting goods to stores</t>
+  </si>
+  <si>
+    <t>To set the salary of every employee</t>
+  </si>
+  <si>
+    <t>A product sold under two different names</t>
+  </si>
+  <si>
+    <t>To explain how the organisation creates, delivers and captures value</t>
+  </si>
+  <si>
+    <t>The duration of an advertising campaign</t>
+  </si>
+  <si>
+    <t>Cash is taxed but profit is not</t>
+  </si>
+  <si>
+    <t>The largest segment in an industry</t>
+  </si>
+  <si>
+    <t>The shared values and norms that shape how people behave at work</t>
+  </si>
+  <si>
+    <t>To define the company's brand colours</t>
+  </si>
+  <si>
+    <t>A fixed legal limit on company size</t>
+  </si>
+  <si>
+    <t>To share customer lists across the industry</t>
+  </si>
+  <si>
+    <t>To set out agreed terms of supply, price and obligations</t>
+  </si>
+  <si>
+    <t>The number of products in the catalogue</t>
+  </si>
+  <si>
+    <t>A specific, longer-term goal that supports the organisation's direction</t>
+  </si>
+  <si>
+    <t>The tax paid against the revenue earned</t>
+  </si>
+  <si>
+    <t>It reduces the number of staff required</t>
+  </si>
+  <si>
+    <t>The time taken to assemble a single unit</t>
+  </si>
+  <si>
+    <t>Offering something customers value that rivals do not match</t>
+  </si>
+  <si>
+    <t>To choose the firm's suppliers</t>
+  </si>
+  <si>
+    <t>To reduce the cost of each unit produced</t>
+  </si>
+  <si>
+    <t>The number of retail outlets it operates</t>
+  </si>
+  <si>
+    <t>Whether a proposed project is practical and worth pursuing</t>
+  </si>
+  <si>
+    <t>It guarantees unanimous decisions</t>
+  </si>
+  <si>
+    <t>The rate at which prices rise</t>
+  </si>
+  <si>
+    <t>To set the selling price of goods</t>
+  </si>
+  <si>
+    <t>How easily assets can be converted into cash</t>
+  </si>
+  <si>
+    <t>To stop competitors from advertising</t>
+  </si>
+  <si>
+    <t>The audience present at a shareholder meeting</t>
+  </si>
+  <si>
+    <t>The period remaining before a patent expires</t>
+  </si>
+  <si>
+    <t>To give shareholders and others an account of performance and position</t>
+  </si>
+  <si>
+    <t>The penalty for cancelling a contract</t>
+  </si>
+  <si>
+    <t>The distribution of salaries within a team</t>
+  </si>
+  <si>
+    <t>Stacking inventory more efficiently in a warehouse</t>
+  </si>
+  <si>
+    <t>It prepares a response in advance for things that may go wrong</t>
+  </si>
+  <si>
+    <t>The total value of unsold stock</t>
+  </si>
+  <si>
+    <t>To transfer ownership of the service</t>
+  </si>
+  <si>
+    <t>To satisfy an annual advertising quota</t>
+  </si>
+  <si>
+    <t>How much demand responds to a change in price</t>
+  </si>
+  <si>
+    <t>The insurance premiums paid annually</t>
+  </si>
+  <si>
+    <t>It fixes the company's production capacity</t>
+  </si>
+  <si>
+    <t>To rank employees for annual appraisal</t>
+  </si>
+  <si>
+    <t>The seating layout of the head office</t>
+  </si>
+  <si>
+    <t>A condition that makes it difficult for new firms to start competing in an industry</t>
+  </si>
+  <si>
+    <t>Every department receives an equal budget</t>
+  </si>
+  <si>
+    <t>Setting one price for every customer</t>
+  </si>
+  <si>
+    <t>The number of patents it holds</t>
+  </si>
+  <si>
+    <t>To fund day-to-day operating needs such as stock and receivables</t>
+  </si>
+  <si>
+    <t>The date on which a loan must be repaid in full</t>
+  </si>
+  <si>
+    <t>To eliminate the need for market research</t>
+  </si>
+  <si>
+    <t>The minimum qualification required of new hires</t>
+  </si>
+  <si>
+    <t>To oversee management and represent shareholders' interests</t>
+  </si>
+  <si>
+    <t>The priority given to senior staff in promotions</t>
+  </si>
+  <si>
+    <t>To rank suppliers by reliability</t>
+  </si>
+  <si>
+    <t>The total spend on advertising last year</t>
+  </si>
+  <si>
+    <t>Have an external provider perform activities it once did in-house</t>
+  </si>
+  <si>
+    <t>A list of a company's shareholders</t>
+  </si>
+  <si>
+    <t>To measure the physical size of a premises</t>
+  </si>
+  <si>
+    <t>A business relocating its head office</t>
+  </si>
+  <si>
+    <t>Operating profit expressed as a percentage of revenue</t>
+  </si>
+  <si>
+    <t>Long-standing customers require no service support</t>
+  </si>
+  <si>
+    <t>A supplier who has signed an exclusivity deal</t>
+  </si>
+  <si>
+    <t>Appointing the target's staff to new roles</t>
+  </si>
+  <si>
+    <t>To test a product with a limited audience before committing to full rollout</t>
+  </si>
+  <si>
+    <t>The cost that is always largest in the accounts</t>
+  </si>
+  <si>
+    <t>Allocates advertising budget between regions</t>
+  </si>
+  <si>
+    <t>To reduce its employee headcount automatically</t>
+  </si>
+  <si>
+    <t>It creates strategic fit and strengthens competitive advantage</t>
+  </si>
+  <si>
+    <t>The forecast demand for next year</t>
+  </si>
+  <si>
+    <t>To register a company with the authorities</t>
+  </si>
+  <si>
+    <t>A longer trading history than competitors</t>
+  </si>
+  <si>
+    <t>How quickly stock is sold and replaced over a period</t>
+  </si>
+  <si>
+    <t>To decide the company's legal structure</t>
+  </si>
+  <si>
+    <t>A meeting between two boards of directors</t>
+  </si>
+  <si>
+    <t>To schedule staff holidays for the year</t>
+  </si>
+  <si>
+    <t>How long it takes to move from idea to a product customers can buy</t>
+  </si>
+  <si>
+    <t>Profit is only calculated when a business closes</t>
+  </si>
+  <si>
+    <t>A market restricted to a single country</t>
+  </si>
+  <si>
+    <t>The company's registered trading name</t>
+  </si>
+  <si>
+    <t>To plan and control the allocation of financial resources</t>
+  </si>
+  <si>
+    <t>The process of reducing a product range</t>
+  </si>
+  <si>
+    <t>To merge reporting systems with competitors</t>
+  </si>
+  <si>
+    <t>To fix the retail price charged to consumers</t>
+  </si>
+  <si>
+    <t>The length of the product warranty</t>
+  </si>
+  <si>
+    <t>A one-off discount offered to a client</t>
+  </si>
+  <si>
+    <t>The gain from an investment against its cost</t>
+  </si>
+  <si>
+    <t>It guarantees faster decisions in every case</t>
+  </si>
+  <si>
+    <t>The recycling process that follows disposal</t>
+  </si>
+  <si>
+    <t>Producing the largest possible volume</t>
+  </si>
+  <si>
+    <t>To define roles, reporting lines and how work is coordinated</t>
+  </si>
+  <si>
+    <t>To satisfy a legal reporting requirement</t>
+  </si>
+  <si>
+    <t>The share price relative to earnings</t>
+  </si>
+  <si>
+    <t>The market value of the company's premises</t>
+  </si>
+  <si>
+    <t>A wider range of perspectives tends to improve problem solving</t>
+  </si>
+  <si>
+    <t>The frequency of board meetings</t>
+  </si>
+  <si>
+    <t>To decide which markets to enter</t>
+  </si>
+  <si>
+    <t>The number of transactions processed per day</t>
+  </si>
+  <si>
+    <t>To expand using partners' capital and local knowledge</t>
+  </si>
+  <si>
+    <t>The staff attending a training session</t>
+  </si>
+  <si>
+    <t>The notice period an employee must serve</t>
+  </si>
+  <si>
+    <t>To negotiate prices with suppliers</t>
+  </si>
+  <si>
+    <t>The value of the next best alternative given up when a choice is made</t>
+  </si>
+  <si>
+    <t>The layout of a factory floor</t>
+  </si>
+  <si>
+    <t>Listing shares on a second exchange</t>
+  </si>
+  <si>
+    <t>It guarantees a project will finish early</t>
+  </si>
+  <si>
+    <t>Revenue less the direct cost of goods sold</t>
+  </si>
+  <si>
+    <t>To register a service as a trademark</t>
+  </si>
+  <si>
+    <t>To increase the company's share capital</t>
+  </si>
+  <si>
+    <t>The difference between cost and selling price</t>
+  </si>
+  <si>
+    <t>Identified risks with their likelihood, impact and planned response</t>
+  </si>
+  <si>
+    <t>It sets the legal jurisdiction for disputes</t>
   </si>
   <si>
     <t>B</t>

</xml_diff>